<commit_message>
Revisao da reuniao 28-09: ramo unico de 24 V, 100 nF a 50 V, um so MPN de 1 uF
- Saem F2, o diodo e o condensador do ramo +24V_ADC; F1 + diodo alimentam o
  R-78HB e o +24V_ADC. +24V_REG deixa de existir (esquematico, PCB, netclasses).
- Condensador de entrada do R-78HB conferido contra o datasheet Recom (p.4):
  10 uF/100 V cumpre os 3,3 uF/100 V pedidos com Vin > 50 V. Sem alteracao.
- 100 nF fora do 24 V -> TDK C1608X7R1H104K080AA (50 V); o do +24V_ADC fica
  GRM188R72A104KA35D (100 V). 1 uF -> TDK C1608X7R1H105K080AB nos quatro.
- Notas 2, 13 e 14 da folha 2; README e registo em 00-Especificacoes;
  catalogo TDK em Documentos_de_Referencia.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KPnkiJQKrkjgRqqw9M78ie
</commit_message>
<xml_diff>
--- a/Desenvolvimento_IC2S-EBM7-2608-V2.3-Fixo420/Arquivos_Fabricação_IC2S-EBM7-2608-V2.3-Fixo420/01-BOM_List_IC2S-EBM7-2608-V2.3-Fixo420/IC2S-EBM7-2608-V2.3-Fixo420-Preliminar.xlsx
+++ b/Desenvolvimento_IC2S-EBM7-2608-V2.3-Fixo420/Arquivos_Fabricação_IC2S-EBM7-2608-V2.3-Fixo420/01-BOM_List_IC2S-EBM7-2608-V2.3-Fixo420/IC2S-EBM7-2608-V2.3-Fixo420-Preliminar.xlsx
@@ -49,9 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -476,9 +479,9 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>C1,C2,C34,C35</t>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>C1,C34,C35</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -497,18 +500,17 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+        <v>3</v>
+      </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>C3,C5</t>
         </is>
@@ -531,7 +533,6 @@
       <c r="F3" t="n">
         <v>2</v>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>2</v>
       </c>
@@ -540,14 +541,14 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>C4,C9,C10,C12,C13,C18,C19,C20,C23,C24,C26,C27,C28,C29,C30,C31,C32,C33,C37,C39,C40,C42,C43,C44</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>100nF/50V</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -557,13 +558,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GRM188R72A104KA35D</t>
+          <t>C1608X7R1H104K080AA</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>24</v>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>24</v>
       </c>
@@ -572,7 +572,7 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>C6,C8,C14,C17,C25,C45</t>
         </is>
@@ -595,7 +595,6 @@
       <c r="F5" t="n">
         <v>6</v>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>6</v>
       </c>
@@ -604,7 +603,7 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>C7,C11,C46</t>
         </is>
@@ -627,7 +626,6 @@
       <c r="F6" t="n">
         <v>3</v>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>3</v>
       </c>
@@ -636,7 +634,7 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>C15,C16</t>
         </is>
@@ -659,7 +657,6 @@
       <c r="F7" t="n">
         <v>2</v>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>2</v>
       </c>
@@ -668,14 +665,14 @@
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>C21</t>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>C21,C22,C41,C47</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1uF</t>
+          <t>1uF/50V</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -685,29 +682,28 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>885012206002</t>
+          <t>C1608X7R1H105K080AB</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>C22</t>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>C36</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1uF</t>
+          <t>100nF/100V</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -717,13 +713,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>C0603C105K4RACTU</t>
+          <t>GRM188R72A104KA35D</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>1</v>
       </c>
@@ -732,30 +727,29 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>C36</t>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>C38</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>100nF/100V</t>
+          <t>10uF/50V</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603C</t>
+          <t>EBM7_V23:C_1206_3216Metric</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>GRM188R72A104KA35D</t>
+          <t>C3216X5R1H106K160AB</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>1</v>
       </c>
@@ -764,30 +758,29 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>C38</t>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>C48</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10uF/50V</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EBM7_V23:C_1206_3216Metric</t>
+          <t>EBM7_V23:0603C</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>C3216X5R1H106K160AB</t>
+          <t>GCM188R71H103KA37J</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>1</v>
       </c>
@@ -796,62 +789,60 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>C41,C47</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1uF/16V</t>
+          <t>SMA6J33A-Q</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603C</t>
+          <t>EBM7_V23:DO-214</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>C0603C105K4RACTU</t>
+          <t>SMA6J33A-Q</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>C48</t>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>MBR1H100SF</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603C</t>
+          <t>EBM7_V23:SOD123</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GCM188R71H103KA37J</t>
+          <t>MBR1H100SFT3G</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>1</v>
       </c>
@@ -860,30 +851,29 @@
       <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>D1</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SMA6J33A-Q</t>
+          <t>ZMM5234B</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EBM7_V23:DO-214</t>
+          <t>EBM7_V23:SOD-80C</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SMA6J33A-Q</t>
+          <t>ZMM5234B</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
         <v>1</v>
       </c>
@@ -892,30 +882,29 @@
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>D2,D3</t>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>D5,D18</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MBR1H100SF</t>
+          <t>KG EELP41.22</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOD123</t>
+          <t>EBM7_V23:0603LED</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MBR1H100SFT3G</t>
+          <t>KG EELP41.22-PHRH-35-A8J8-20-R18</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>2</v>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>2</v>
       </c>
@@ -924,190 +913,184 @@
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>D4</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>D6,D7,D8,D11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ZMM5234B</t>
+          <t>824500301</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOD-80C</t>
+          <t>EBM7_V23:DO-214</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ZMM5234B</t>
+          <t>824500301</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>D5,D18</t>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>D9,D10,D12,D13</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KG EELP41.22</t>
+          <t>SMBJ36A</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603LED</t>
+          <t>EBM7_V23:DO-214AA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>KG EELP41.22-PHRH-35-A8J8-20-R18</t>
+          <t>SMBJ36A-13-F</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>D6,D7,D8,D11</t>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>D14,D15,D16,D17,D22,D24,D25</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>824500301</t>
+          <t>BAV199</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EBM7_V23:DO-214</t>
+          <t>EBM7_V23:SOT23-3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>824500301</t>
+          <t>BAV199LT1G</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
+        <v>7</v>
+      </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>D9,D10,D12,D13</t>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>D19</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SMBJ36A</t>
+          <t>SMA6J6.0A</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>EBM7_V23:DO-214AA</t>
+          <t>EBM7_V23:DO-214</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SMBJ36A-13-F</t>
+          <t>SMA6J6.0A</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>4</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>D14,D15,D16,D17,D22,D24,D25</t>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>D20,D21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BAV199</t>
+          <t>824500101</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT23-3</t>
+          <t>EBM7_V23:DO-214</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BAV199LT1G</t>
+          <t>824500101</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>7</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>D19</t>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>D23</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SMA6J6.0A</t>
+          <t>RB162MM-60</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>EBM7_V23:DO-214</t>
+          <t>EBM7_V23:SOD-123F</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SMA6J6.0A</t>
+          <t>RB162MM-60TR</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>1</v>
       </c>
@@ -1116,190 +1099,184 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>D20,D21</t>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>F1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>824500101</t>
+          <t>CC12H750MA-TR</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>EBM7_V23:DO-214</t>
+          <t>EBM7_V23:1206F</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>824500101</t>
+          <t>CC12H750MA-TR</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>D23</t>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>F3,F4,F5,F6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>RB162MM-60</t>
+          <t>3413.0006.22</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOD-123F</t>
+          <t>EBM7_V23:1206F</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RB162MM-60TR</t>
+          <t>3413.0006.22</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>F1,F2</t>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>FB1,FB2,FB3,FB4,FB5,FB6,FB7</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CC12H750MA-TR</t>
+          <t>470R@100MHz</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>EBM7_V23:1206F</t>
+          <t>EBM7_V23:0603FB</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CC12H750MA-TR</t>
+          <t>BLM18PG471SN1D</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
+        <v>7</v>
+      </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>F3,F4,F5,F6</t>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>H1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>3413.0006.22</t>
+          <t>FTS-103-01-L-D</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EBM7_V23:1206F</t>
+          <t>EBM7_V23:HDR2X3_1.27mm-Without_number</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>3413.0006.22</t>
+          <t>FTS-103-01-L-D</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>FB1,FB2,FB3,FB4,FB5,FB6,FB7</t>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>470R@100MHz</t>
+          <t>M20-7822046</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603FB</t>
+          <t>EBM7_V23:HDR1X20_FEMALE</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BLM18PG471SN1D</t>
+          <t>M20-7822046</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>7</v>
-      </c>
-      <c r="G26" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H26" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>H1</t>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FTS-103-01-L-D</t>
+          <t>M20-7821446</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>EBM7_V23:HDR2X3_1.27mm-Without_number</t>
+          <t>EBM7_V23:HDR1X14_FEMALE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FTS-103-01-L-D</t>
+          <t>M20-7821446</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
         <v>1</v>
       </c>
@@ -1308,62 +1285,60 @@
       <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>R2,R3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>M20-7822046</t>
+          <t>220R</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EBM7_V23:HDR1X20_FEMALE</t>
+          <t>EBM7_V23:1206R</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>M20-7822046</t>
+          <t>RC1206FR-07220RL</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>R4</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>M20-7821446</t>
+          <t>2k2</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EBM7_V23:HDR1X14_FEMALE</t>
+          <t>EBM7_V23:0603R</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>M20-7821446</t>
+          <t>RC0603FR-072K2L</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
         <v>1</v>
       </c>
@@ -1372,46 +1347,45 @@
       <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>R2,R3</t>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>R5</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>220R</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EBM7_V23:1206R</t>
+          <t>EBM7_V23:0603R</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>RC1206FR-07220RL</t>
+          <t>CRCW0603100KFKEA</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>R4</t>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>R6</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2k2</t>
+          <t>4k42</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1421,13 +1395,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>RC0603FR-072K2L</t>
+          <t>RMCF0603FT4K42</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
         <v>1</v>
       </c>
@@ -1436,14 +1409,14 @@
       <c r="A32" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>R5</t>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>R7,R9,R26</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1453,29 +1426,28 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CRCW0603100KFKEA</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
+        <v>3</v>
+      </c>
       <c r="H32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>R6</t>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>R8</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>4k42</t>
+          <t>0R</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1485,29 +1457,33 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>RMCF0603FT4K42</t>
+          <t>RC0603JR-070RL</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>R7,R9,R26</t>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>R10,R11,R12,R16</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>0R</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1517,29 +1493,28 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603JR-070RL</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
-      </c>
-      <c r="G34" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>R8</t>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>R13,R14,R15,R17</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0R</t>
+          <t>110R</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1549,33 +1524,28 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>RC0603JR-070RL</t>
+          <t>RG1608P-111-B-T5</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>DNP</t>
-        </is>
+        <v>4</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>R10,R11,R12,R16</t>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>R18,R19,R20,R21</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0R</t>
+          <t>3k3</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1585,13 +1555,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>RC0603JR-070RL</t>
+          <t>RC0603FR-073K3L</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>4</v>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
         <v>4</v>
       </c>
@@ -1600,14 +1569,14 @@
       <c r="A37" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>R13,R14,R15,R17</t>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>R22</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>11k5</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1617,29 +1586,28 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>RG1608P-111-B-T5</t>
+          <t>RC0603FR-0711K5L</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4</v>
-      </c>
-      <c r="G37" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>R18,R19,R20,R21</t>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>R23,R24</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3k3</t>
+          <t>6k65</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1649,29 +1617,28 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>RC0603FR-073K3L</t>
+          <t>RC0603FR-076K65L</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4</v>
-      </c>
-      <c r="G38" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>R22</t>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>R25</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>11k5</t>
+          <t>93k1</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1681,13 +1648,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>RC0603FR-0711K5L</t>
+          <t>RMCF0603FT93K1</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
         <v>1</v>
       </c>
@@ -1696,14 +1662,14 @@
       <c r="A40" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>R23,R24</t>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>R27</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>6k65</t>
+          <t>22k</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1713,29 +1679,28 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>RC0603FR-076K65L</t>
+          <t>ERJ-3EKF2202V</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
-      </c>
-      <c r="G40" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>R25</t>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>R28,R29</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>93k1</t>
+          <t>10k 0.1%</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1745,45 +1710,43 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>RMCF0603FT93K1</t>
+          <t>RG1608P-103-B-T5</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>R27</t>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>R30</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>22k</t>
+          <t>68R 1W</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603R</t>
+          <t>EBM7_V23:1206R</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ERJ-3EKF2202V</t>
+          <t>SG73P2BTTD68R0F</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
         <v>1</v>
       </c>
@@ -1792,14 +1755,14 @@
       <c r="A43" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>R28,R29</t>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>R31,R32</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>10k 0.1%</t>
+          <t>1k3 0.1%</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1809,13 +1772,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>RG1608P-103-B-T5</t>
+          <t>RG1608P-132-B-T5</t>
         </is>
       </c>
       <c r="F43" t="n">
         <v>2</v>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
         <v>2</v>
       </c>
@@ -1824,30 +1786,29 @@
       <c r="A44" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>R30</t>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>R36</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>68R 1W</t>
+          <t>NTC 10k</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>EBM7_V23:1206R</t>
+          <t>EBM7_V23:0603R</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SG73P2BTTD68R0F</t>
+          <t>NTCS0603E3103JLT</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
         <v>1</v>
       </c>
@@ -1856,14 +1817,14 @@
       <c r="A45" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>R31,R32</t>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>R37</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1k3 0.1%</t>
+          <t>22k 0.1%</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1873,29 +1834,28 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>RG1608P-132-B-T5</t>
+          <t>RG1608P-223-B-T5</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>2</v>
-      </c>
-      <c r="G45" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>R36</t>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>R38,R39</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>NTC 10k</t>
+          <t>3k</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1905,45 +1865,43 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>NTCS0603E3103JLT</t>
+          <t>RC0603FR-073KL</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" t="inlineStr"/>
+        <v>2</v>
+      </c>
       <c r="H46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>R37</t>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>U1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>22k 0.1%</t>
+          <t>R-78HB5.0-0.5L</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603R</t>
+          <t>EBM7_V23:R-78HBxx-0.5L_SIP-3H</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>RG1608P-223-B-T5</t>
+          <t>R-78HB5.0-0.5L</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
         <v>1</v>
       </c>
@@ -1952,62 +1910,60 @@
       <c r="A48" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>R38,R39</t>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>U2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>3k</t>
+          <t>MCP1824ST-3302E/DB</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EBM7_V23:0603R</t>
+          <t>EBM7_V23:SOT-223-3</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>RC0603FR-073KL</t>
+          <t>MCP1824ST-3302E/DB</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>2</v>
-      </c>
-      <c r="G48" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>U1</t>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>U3</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>R-78HB5.0-0.5L</t>
+          <t>SPX3819M5-L-3-3/TR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>EBM7_V23:R-78HBxx-0.5L_SIP-3H</t>
+          <t>EBM7_V23:SOT-23-5</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>R-78HB5.0-0.5L</t>
+          <t>SPX3819M5-L-3-3/TR</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>1</v>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
         <v>1</v>
       </c>
@@ -2016,30 +1972,29 @@
       <c r="A50" t="n">
         <v>49</v>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>U2</t>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>U4</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>MCP1824ST-3302E/DB</t>
+          <t>TL431B</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT-223-3</t>
+          <t>EBM7_V23:SOT23-3</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>MCP1824ST-3302E/DB</t>
+          <t>TL431BQDBZR</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>1</v>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
         <v>1</v>
       </c>
@@ -2048,30 +2003,29 @@
       <c r="A51" t="n">
         <v>50</v>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>U3</t>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>U5</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SPX3819M5-L-3-3/TR</t>
+          <t>ISO7141CCDBQR</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT-23-5</t>
+          <t>EBM7_V23:SSOP16-4.9x3.9mm</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SPX3819M5-L-3-3/TR</t>
+          <t>ISO7141CCDBQR</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="n">
         <v>1</v>
       </c>
@@ -2080,30 +2034,29 @@
       <c r="A52" t="n">
         <v>51</v>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>U4</t>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>U6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TL431B</t>
+          <t>AD7124-8BCPZ</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT23-3</t>
+          <t>EBM7_V23:LFCSP-32-2</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TL431BQDBZR</t>
+          <t>AD7124-8BCPZ</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
         <v>1</v>
       </c>
@@ -2112,30 +2065,29 @@
       <c r="A53" t="n">
         <v>52</v>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>U5</t>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>U7</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ISO7141CCDBQR</t>
+          <t>ADR4525BRZ</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>EBM7_V23:SSOP16-4.9x3.9mm</t>
+          <t>EBM7_V23:SOIC8</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ISO7141CCDBQR</t>
+          <t>ADR4525BRZ</t>
         </is>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
         <v>1</v>
       </c>
@@ -2144,62 +2096,60 @@
       <c r="A54" t="n">
         <v>53</v>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>U6</t>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>U8,U9,U10,U11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>AD7124-8BCPZ</t>
+          <t>TPS26613DDFR</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>EBM7_V23:LFCSP-32-2</t>
+          <t>EBM7_V23:SOT-23-8</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>AD7124-8BCPZ</t>
+          <t>TPS26613DDFR</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>1</v>
-      </c>
-      <c r="G54" t="inlineStr"/>
+        <v>4</v>
+      </c>
       <c r="H54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
         <v>54</v>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>U7</t>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>U12</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ADR4525BRZ</t>
+          <t>TPS7A4001DGN</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOIC8</t>
+          <t>EBM7_V23:HVSSOP-8-1EP</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ADR4525BRZ</t>
+          <t>TPS7A4001DGNR</t>
         </is>
       </c>
       <c r="F55" t="n">
         <v>1</v>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
         <v>1</v>
       </c>
@@ -2208,103 +2158,40 @@
       <c r="A56" t="n">
         <v>55</v>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>U8,U9,U10,U11</t>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>U13</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>TPS26613DDFR</t>
+          <t>LP5907MFX-2.5</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT-23-8</t>
+          <t>EBM7_V23:SOT-23-5</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>TPS26613DDFR</t>
+          <t>LP5907MFX-2.5/NOPB</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>4</v>
-      </c>
-      <c r="G56" t="inlineStr"/>
+        <v>1</v>
+      </c>
       <c r="H56" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>U12</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>TPS7A4001DGN</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>EBM7_V23:HVSSOP-8-1EP</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>TPS7A4001DGNR</t>
-        </is>
-      </c>
-      <c r="F57" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="n">
-        <v>1</v>
-      </c>
+      <c r="B57" s="2" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>LP5907MFX-2.5</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>EBM7_V23:SOT-23-5</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>LP5907MFX-2.5/NOPB</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>1</v>
-      </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>PRELIMINAR - placa ainda sem revisao independente do roteamento (2shw-pcb:check-roteamento). Gerado do esquematico em 25-09-2026.</t>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>PRELIMINAR - placa ainda sem revisao independente do roteamento (2shw-pcb:check-roteamento). Gerado do esquematico em 28-09-2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LDO 3,3 V do lado PLC: U2 MCP1824ST (SOT-223) -> SPX3819M5-L-3-3/TR (SOT-23-5), mesmo MPN do U3
- Criterio da equipa: menos MPN, mais pecas do mesmo tipo; o MCP1824ST sai.
- EN a VIN, BYP aberto; estabilidade com ceramico sem garantia no datasheet (provada em campo na V2.2).
- Esquematico: ERC 0; netlist so muda os pinos do U2. PCB: pegada SOT-23-5 no
  mesmo sitio; faltam rotear 6 ligacoes do U2; Gerbers/PnP por regenerar depois.
- Registo: alteracao_LDO_3V3_lado_PLC_2026-09-28.md (comparacao, verificacao e
  riscos em aberto). BOM e PDF do esquematico regenerados.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KPnkiJQKrkjgRqqw9M78ie
</commit_message>
<xml_diff>
--- a/Desenvolvimento_IC2S-EBM7-2608-V2.3-Fixo420/Arquivos_Fabricação_IC2S-EBM7-2608-V2.3-Fixo420/01-BOM_List_IC2S-EBM7-2608-V2.3-Fixo420/IC2S-EBM7-2608-V2.3-Fixo420-Preliminar.xlsx
+++ b/Desenvolvimento_IC2S-EBM7-2608-V2.3-Fixo420/Arquivos_Fabricação_IC2S-EBM7-2608-V2.3-Fixo420/01-BOM_List_IC2S-EBM7-2608-V2.3-Fixo420/IC2S-EBM7-2608-V2.3-Fixo420-Preliminar.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1912,29 +1912,29 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U2,U3</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>MCP1824ST-3302E/DB</t>
+          <t>SPX3819M5-L-3-3/TR</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT-223-3</t>
+          <t>EBM7_V23:SOT-23-5</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>MCP1824ST-3302E/DB</t>
+          <t>SPX3819M5-L-3-3/TR</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -1943,22 +1943,22 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SPX3819M5-L-3-3/TR</t>
+          <t>TL431B</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT-23-5</t>
+          <t>EBM7_V23:SOT23-3</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>SPX3819M5-L-3-3/TR</t>
+          <t>TL431BQDBZR</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -1974,22 +1974,22 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>TL431B</t>
+          <t>ISO7141CCDBQR</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT23-3</t>
+          <t>EBM7_V23:SSOP16-4.9x3.9mm</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>TL431BQDBZR</t>
+          <t>ISO7141CCDBQR</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2005,22 +2005,22 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ISO7141CCDBQR</t>
+          <t>AD7124-8BCPZ</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>EBM7_V23:SSOP16-4.9x3.9mm</t>
+          <t>EBM7_V23:LFCSP-32-2</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ISO7141CCDBQR</t>
+          <t>AD7124-8BCPZ</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -2036,22 +2036,22 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U7</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AD7124-8BCPZ</t>
+          <t>ADR4525BRZ</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>EBM7_V23:LFCSP-32-2</t>
+          <t>EBM7_V23:SOIC8</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>AD7124-8BCPZ</t>
+          <t>ADR4525BRZ</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -2067,29 +2067,29 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U8,U9,U10,U11</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ADR4525BRZ</t>
+          <t>TPS26613DDFR</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOIC8</t>
+          <t>EBM7_V23:SOT-23-8</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ADR4525BRZ</t>
+          <t>TPS26613DDFR</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54">
@@ -2098,29 +2098,29 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>U8,U9,U10,U11</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>TPS26613DDFR</t>
+          <t>TPS7A4001DGN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>EBM7_V23:SOT-23-8</t>
+          <t>EBM7_V23:HVSSOP-8-1EP</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>TPS26613DDFR</t>
+          <t>TPS7A4001DGNR</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -2129,22 +2129,22 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>TPS7A4001DGN</t>
+          <t>LP5907MFX-2.5</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>EBM7_V23:HVSSOP-8-1EP</t>
+          <t>EBM7_V23:SOT-23-5</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>TPS7A4001DGNR</t>
+          <t>LP5907MFX-2.5/NOPB</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -2155,41 +2155,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>LP5907MFX-2.5</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>EBM7_V23:SOT-23-5</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>LP5907MFX-2.5/NOPB</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>1</v>
-      </c>
-      <c r="H56" t="n">
-        <v>1</v>
-      </c>
+      <c r="B56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="2" t="n"/>
-    </row>
-    <row r="58">
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>PRELIMINAR - placa ainda sem revisao independente do roteamento (2shw-pcb:check-roteamento). Gerado do esquematico em 28-09-2026.</t>
         </is>

</xml_diff>

<commit_message>
C49 2,2 uF na saida do U2 (SPX3819), como a saida do SPX da V2.2 em campo
- Datasheet SPX3819 Fig. 18 (p.8) conferido: EN a VIN e BYP aberto como a figura; saida
  cerâmica 2,2 + 10 uF + 100 nF (V2.2 so tinha ceramicos no SPX). MPN C1608X5R1E225K080AB
  ja na BOM (C7/C11/C46). PCB: clone do C8 a 3 mm do U2, 2 ligacoes por rotear.
- Inclui as alteracoes de roteamento em curso do projectista no PCB.
- ERC 0; DRC 0 erros, sem avisos novos, paridade 0. BOM e PDF regenerados.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KPnkiJQKrkjgRqqw9M78ie
</commit_message>
<xml_diff>
--- a/Desenvolvimento_IC2S-EBM7-2608-V2.3-Fixo420/Arquivos_Fabricação_IC2S-EBM7-2608-V2.3-Fixo420/01-BOM_List_IC2S-EBM7-2608-V2.3-Fixo420/IC2S-EBM7-2608-V2.3-Fixo420-Preliminar.xlsx
+++ b/Desenvolvimento_IC2S-EBM7-2608-V2.3-Fixo420/Arquivos_Fabricação_IC2S-EBM7-2608-V2.3-Fixo420/01-BOM_List_IC2S-EBM7-2608-V2.3-Fixo420/IC2S-EBM7-2608-V2.3-Fixo420-Preliminar.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>C7,C11,C46</t>
+          <t>C7,C11,C46,C49</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">

</xml_diff>